<commit_message>
feat(content-runtime): G01-P7-M09 compile authored hit formulas
</commit_message>
<xml_diff>
--- a/config/generated/templates/AbilityHitPlanBinding.xlsx
+++ b/config/generated/templates/AbilityHitPlanBinding.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
   <si>
     <t>@table</t>
   </si>
@@ -40,7 +40,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>dbb2c00ed65aabfb</t>
+    <t>4b2940e76849c763</t>
   </si>
   <si>
     <t>#name</t>
@@ -55,6 +55,21 @@
     <t>hit_plan_id</t>
   </si>
   <si>
+    <t>damage_parameter_key</t>
+  </si>
+  <si>
+    <t>damage_scaling_stat</t>
+  </si>
+  <si>
+    <t>damage_class</t>
+  </si>
+  <si>
+    <t>element</t>
+  </si>
+  <si>
+    <t>base_toughness_decimal</t>
+  </si>
+  <si>
     <t>#field</t>
   </si>
   <si>
@@ -70,6 +85,18 @@
     <t>ref&lt;HitPlan.id&gt;</t>
   </si>
   <si>
+    <t>optional&lt;string&gt;</t>
+  </si>
+  <si>
+    <t>optional&lt;enum&lt;HitScalingStat&gt;&gt;</t>
+  </si>
+  <si>
+    <t>optional&lt;enum&lt;HitDamageClass&gt;&gt;</t>
+  </si>
+  <si>
+    <t>optional&lt;enum&lt;HitElement&gt;&gt;</t>
+  </si>
+  <si>
     <t>#scope</t>
   </si>
   <si>
@@ -77,6 +104,9 @@
   </si>
   <si>
     <t>range=1..100</t>
+  </si>
+  <si>
+    <t>length=1..32</t>
   </si>
   <si>
     <t>#desc</t>
@@ -503,6 +533,10 @@
     <col min="2" max="2" width="15.7109375" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" style="5" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="30.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="26.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -548,10 +582,25 @@
       <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>10</v>
@@ -561,25 +610,55 @@
       </c>
       <c r="D3" s="5" t="s">
         <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
@@ -588,32 +667,68 @@
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="4">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 100." promptTitle="Integer range" prompt="Enter an integer from 1 to 100." sqref="C8:C1007">
       <formula1>1</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Atk, Hp, Def" promptTitle="HitScalingStat enum" prompt="Select a value from the dropdown." sqref="F8:F1007">
+      <formula1>"Atk,Hp,Def"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Ordinary, Dot, Additional, Elation" promptTitle="HitDamageClass enum" prompt="Select a value from the dropdown." sqref="G8:G1007">
+      <formula1>"Ordinary,Dot,Additional,Elation"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Physical, Fire, Ice, Lightning, Wind, Quantum, Imaginary" promptTitle="HitElement enum" prompt="Select a value from the dropdown." sqref="H8:H1007">
+      <formula1>"Physical,Fire,Ice,Lightning,Wind,Quantum,Imaginary"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>